<commit_message>
make the CAM escalation dynamic
</commit_message>
<xml_diff>
--- a/artifacts/Rental Specimen.xlsx
+++ b/artifacts/Rental Specimen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0050s8t\Documents\rental-automation\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D6D59E-07E5-409D-9B8A-8CB82AB8DFCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68731A05-8D14-4278-9705-47D3B10FAA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="764" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="764" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="16" state="hidden" r:id="rId1"/>
@@ -170,7 +170,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="502">
   <si>
     <t>RENTAL CALCULATION FOR NEW LEASE</t>
   </si>
@@ -1757,6 +1757,14 @@
   </si>
   <si>
     <t>PM per sq. mtr. per month</t>
+  </si>
+  <si>
+    <t>Rental 
+SQF</t>
+  </si>
+  <si>
+    <t>CAM 
+SQF</t>
   </si>
 </sst>
 </file>
@@ -26632,10 +26640,10 @@
         <v>66</v>
       </c>
       <c r="K30" s="590" t="s">
-        <v>252</v>
+        <v>500</v>
       </c>
       <c r="L30" s="590" t="s">
-        <v>254</v>
+        <v>501</v>
       </c>
       <c r="M30" s="591" t="s">
         <v>29</v>
@@ -26685,11 +26693,11 @@
         <v>1141800</v>
       </c>
       <c r="L31" s="481">
-        <f t="shared" ref="L31:L62" si="27">J31*E31</f>
+        <f>J31*E31</f>
         <v>147292.20000000001</v>
       </c>
       <c r="M31" s="483">
-        <f t="shared" ref="M31:M36" si="28">I31+K31+L31</f>
+        <f t="shared" ref="M31:M36" si="27">I31+K31+L31</f>
         <v>1289092.2</v>
       </c>
       <c r="N31" s="501"/>
@@ -26732,11 +26740,11 @@
         <v>1141800</v>
       </c>
       <c r="L32" s="486">
+        <f t="shared" ref="L31:L62" si="28">J32*E32</f>
+        <v>147292.20000000001</v>
+      </c>
+      <c r="M32" s="467">
         <f t="shared" si="27"/>
-        <v>147292.20000000001</v>
-      </c>
-      <c r="M32" s="467">
-        <f t="shared" si="28"/>
         <v>1289092.2</v>
       </c>
       <c r="N32" s="465"/>
@@ -26782,11 +26790,11 @@
         <v>1141800</v>
       </c>
       <c r="L33" s="486">
+        <f t="shared" si="28"/>
+        <v>147292.20000000001</v>
+      </c>
+      <c r="M33" s="467">
         <f t="shared" si="27"/>
-        <v>147292.20000000001</v>
-      </c>
-      <c r="M33" s="467">
-        <f t="shared" si="28"/>
         <v>1289092.2</v>
       </c>
       <c r="N33" s="465"/>
@@ -26832,11 +26840,11 @@
         <v>1141800</v>
       </c>
       <c r="L34" s="486">
+        <f t="shared" si="28"/>
+        <v>147292.20000000001</v>
+      </c>
+      <c r="M34" s="467">
         <f t="shared" si="27"/>
-        <v>147292.20000000001</v>
-      </c>
-      <c r="M34" s="467">
-        <f t="shared" si="28"/>
         <v>1289092.2</v>
       </c>
       <c r="N34" s="465"/>
@@ -26882,11 +26890,11 @@
         <v>1141800</v>
       </c>
       <c r="L35" s="486">
+        <f t="shared" si="28"/>
+        <v>147292.20000000001</v>
+      </c>
+      <c r="M35" s="467">
         <f t="shared" si="27"/>
-        <v>147292.20000000001</v>
-      </c>
-      <c r="M35" s="467">
-        <f t="shared" si="28"/>
         <v>1289092.2</v>
       </c>
       <c r="N35" s="465"/>
@@ -26932,11 +26940,11 @@
         <v>1141800</v>
       </c>
       <c r="L36" s="486">
+        <f t="shared" si="28"/>
+        <v>147292.20000000001</v>
+      </c>
+      <c r="M36" s="467">
         <f t="shared" si="27"/>
-        <v>147292.20000000001</v>
-      </c>
-      <c r="M36" s="467">
-        <f t="shared" si="28"/>
         <v>1289092.2</v>
       </c>
       <c r="N36" s="465"/>
@@ -26981,7 +26989,7 @@
         <v>1141800</v>
       </c>
       <c r="L37" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>147292.20000000001</v>
       </c>
       <c r="M37" s="467">
@@ -27031,7 +27039,7 @@
         <v>1141800</v>
       </c>
       <c r="L38" s="491">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>147292.20000000001</v>
       </c>
       <c r="M38" s="493">
@@ -27080,7 +27088,7 @@
         <v>1141800</v>
       </c>
       <c r="L39" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>147292.20000000001</v>
       </c>
       <c r="M39" s="467">
@@ -27135,7 +27143,7 @@
         <v>1141800</v>
       </c>
       <c r="L40" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>147292.20000000001</v>
       </c>
       <c r="M40" s="467">
@@ -27184,7 +27192,7 @@
         <v>1141800</v>
       </c>
       <c r="L41" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>147292.20000000001</v>
       </c>
       <c r="M41" s="467">
@@ -27233,7 +27241,7 @@
         <v>1141800</v>
       </c>
       <c r="L42" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>147292.20000000001</v>
       </c>
       <c r="M42" s="467">
@@ -27282,7 +27290,7 @@
         <v>1141800</v>
       </c>
       <c r="L43" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M43" s="467">
@@ -27331,7 +27339,7 @@
         <v>1141800</v>
       </c>
       <c r="L44" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M44" s="467">
@@ -27380,7 +27388,7 @@
         <v>1141800</v>
       </c>
       <c r="L45" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M45" s="467">
@@ -27429,7 +27437,7 @@
         <v>1141800</v>
       </c>
       <c r="L46" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M46" s="467">
@@ -27478,7 +27486,7 @@
         <v>1141800</v>
       </c>
       <c r="L47" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M47" s="467">
@@ -27527,7 +27535,7 @@
         <v>1141800</v>
       </c>
       <c r="L48" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M48" s="467">
@@ -27576,7 +27584,7 @@
         <v>1141800</v>
       </c>
       <c r="L49" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M49" s="467">
@@ -27626,7 +27634,7 @@
         <v>1141800</v>
       </c>
       <c r="L50" s="491">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M50" s="493">
@@ -27675,7 +27683,7 @@
         <v>1141800</v>
       </c>
       <c r="L51" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M51" s="467">
@@ -27730,7 +27738,7 @@
         <v>1141800</v>
       </c>
       <c r="L52" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M52" s="467">
@@ -27779,7 +27787,7 @@
         <v>1141800</v>
       </c>
       <c r="L53" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M53" s="467">
@@ -27828,7 +27836,7 @@
         <v>1141800</v>
       </c>
       <c r="L54" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>154656.81000000003</v>
       </c>
       <c r="M54" s="467">
@@ -27877,7 +27885,7 @@
         <v>1141800</v>
       </c>
       <c r="L55" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M55" s="467">
@@ -27926,7 +27934,7 @@
         <v>1141800</v>
       </c>
       <c r="L56" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M56" s="467">
@@ -27975,7 +27983,7 @@
         <v>1141800</v>
       </c>
       <c r="L57" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M57" s="467">
@@ -28024,7 +28032,7 @@
         <v>1141800</v>
       </c>
       <c r="L58" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M58" s="467">
@@ -28073,7 +28081,7 @@
         <v>1141800</v>
       </c>
       <c r="L59" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M59" s="467">
@@ -28122,7 +28130,7 @@
         <v>1141800</v>
       </c>
       <c r="L60" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M60" s="467">
@@ -28171,7 +28179,7 @@
         <v>1141800</v>
       </c>
       <c r="L61" s="486">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M61" s="467">
@@ -28221,7 +28229,7 @@
         <v>1141800</v>
       </c>
       <c r="L62" s="491">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>162389.65050000002</v>
       </c>
       <c r="M62" s="493">

</xml_diff>

<commit_message>
added the OpEx configuration
</commit_message>
<xml_diff>
--- a/artifacts/Rental Specimen.xlsx
+++ b/artifacts/Rental Specimen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0050s8t\Documents\rental-automation\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C3A8A9-88EB-4D95-BDA7-DB707B27E21A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC8A485-B31D-4E94-A60E-78814B00A0D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="764" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,64 +42,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>in219907</author>
-  </authors>
-  <commentList>
-    <comment ref="G191" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>in219907:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Assumed that Agreement will be of 10yrs hence MV tkn @ 25% which wil be devided equally over a period of 10yrs</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J191" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>in219907:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Assumed that Agreement will be of 10yrs hence MV tkn @ 25% which wil be devided equally over a period of 10yrs</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1272,7 +1214,7 @@
     <numFmt numFmtId="231" formatCode="\V\F\ \ #\-#\-##"/>
     <numFmt numFmtId="232" formatCode="00"/>
   </numFmts>
-  <fonts count="104">
+  <fonts count="102">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1348,19 +1290,6 @@
       <b/>
       <sz val="10"/>
       <name val="Arial Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
@@ -3171,42 +3100,42 @@
   </borders>
   <cellStyleXfs count="1012">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="4" fontId="46" fillId="2" borderId="1">
+    <xf numFmtId="4" fontId="44" fillId="2" borderId="1">
       <alignment readingOrder="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="175" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="175" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="19" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="21" fillId="0" borderId="2">
+    <xf numFmtId="177" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="177" fontId="19" fillId="0" borderId="2">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -3219,10 +3148,10 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="181" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -3233,70 +3162,70 @@
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="37" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="35" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="182" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="179" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="40" fontId="25" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="40" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="37" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="35" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -3310,47 +3239,47 @@
     <xf numFmtId="184" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="184" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="185" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="177" fontId="26" fillId="0" borderId="3" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="185" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="177" fontId="24" fillId="0" borderId="3" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="186" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyProtection="0"/>
-    <xf numFmtId="178" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
-    <xf numFmtId="2" fontId="27" fillId="0" borderId="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="186" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyProtection="0"/>
+    <xf numFmtId="178" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="2" fontId="25" fillId="0" borderId="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="29" fillId="0" borderId="5">
+    <xf numFmtId="168" fontId="27" fillId="0" borderId="5">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="38" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -3359,20 +3288,20 @@
     </xf>
     <xf numFmtId="10" fontId="5" fillId="4" borderId="8" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="177" fontId="10" fillId="5" borderId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="37" fontId="34" fillId="0" borderId="0"/>
-    <xf numFmtId="187" fontId="35" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="37" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="187" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -3380,9 +3309,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -3390,95 +3319,95 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="175" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="175" fontId="48" fillId="0" borderId="0"/>
-    <xf numFmtId="175" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="175" fontId="46" fillId="0" borderId="0"/>
+    <xf numFmtId="175" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="37" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="35" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="48" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="46" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyFont="0"/>
-    <xf numFmtId="188" fontId="37" fillId="5" borderId="0"/>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyFont="0"/>
+    <xf numFmtId="188" fontId="35" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="9">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="1" borderId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="1" borderId="10">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="6" borderId="8">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="6" borderId="9">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="1" borderId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="1" borderId="10">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="6" borderId="8">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="189" fontId="38" fillId="0" borderId="0">
+    <xf numFmtId="189" fontId="36" fillId="0" borderId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
       <alignment horizontal="centerContinuous" vertical="top"/>
     </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="0" applyBorder="0">
+    <xf numFmtId="1" fontId="19" fillId="0" borderId="0" applyBorder="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
-    <xf numFmtId="40" fontId="43" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="40" fontId="41" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="190" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="49" fontId="45" fillId="7" borderId="0">
+    <xf numFmtId="49" fontId="43" fillId="7" borderId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -3519,10 +3448,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="53" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="51" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="57" fillId="3" borderId="1" applyNumberFormat="0">
+    <xf numFmtId="0" fontId="55" fillId="3" borderId="1" applyNumberFormat="0">
       <alignment readingOrder="1"/>
       <protection locked="0"/>
     </xf>
@@ -3547,257 +3476,257 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="8">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="56" fillId="20" borderId="61" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="54" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="54" fillId="20" borderId="61" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="53" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="53" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="51" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="51" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="193" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="194" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="40" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="38" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="195" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="61" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="59" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="1" fontId="5" fillId="45" borderId="62">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="196" fontId="5" fillId="45" borderId="63">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="62" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="62" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="62" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="62" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="62" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="63" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="63" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="197" fontId="56" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="0" fontId="64" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="64" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="64" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="64" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="64" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="64" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="64" fillId="22" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="64" fillId="22" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="65" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="66" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="60" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="60" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="60" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="60" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="60" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="60" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="197" fontId="54" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="62" fillId="22" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="62" fillId="22" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="64" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="198" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="67" fillId="0" borderId="0" applyNumberFormat="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="0" applyNumberFormat="0" applyAlignment="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="199" fontId="68" fillId="47" borderId="0" applyFill="0">
+    <xf numFmtId="199" fontId="66" fillId="47" borderId="0" applyFill="0">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -3806,7 +3735,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="200" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="202" fontId="69" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
+    <xf numFmtId="202" fontId="67" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -3818,22 +3747,22 @@
     <xf numFmtId="208" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="209" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="210" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="70" fillId="0" borderId="0" applyNumberFormat="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" applyNumberFormat="0" applyAlignment="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="211" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="211" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="212" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="212" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="213" fontId="4" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
@@ -3855,7 +3784,7 @@
     <xf numFmtId="213" fontId="4" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="214" fontId="69" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="214" fontId="67" fillId="0" borderId="0" applyFont="0">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -3865,342 +3794,342 @@
     <xf numFmtId="218" fontId="5" fillId="45" borderId="63">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="72" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="199" fontId="73" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="70" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="199" fontId="71" fillId="0" borderId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="74" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="75" fillId="0" borderId="66" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="75" fillId="0" borderId="66" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="79" fillId="0" borderId="69" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="79" fillId="0" borderId="69" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="79" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="79" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="199" fontId="69" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="65" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="73" fillId="0" borderId="66" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="73" fillId="0" borderId="66" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="75" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="75" fillId="0" borderId="67" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="68" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="69" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="69" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="24" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="199" fontId="67" fillId="0" borderId="0" applyFont="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="199" fontId="69" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
+    <xf numFmtId="199" fontId="67" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="40" fontId="5" fillId="0" borderId="0" applyFont="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="199" fontId="69" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="70" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="199" fontId="67" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="199" fontId="69" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
+    <xf numFmtId="199" fontId="67" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="202" fontId="82" fillId="0" borderId="0">
+    <xf numFmtId="202" fontId="80" fillId="0" borderId="0">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="202" fontId="5" fillId="0" borderId="0" applyFont="0"/>
-    <xf numFmtId="41" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="54" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="219" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="4" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="199" fontId="69" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
+    <xf numFmtId="4" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="199" fontId="67" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="83" fillId="0" borderId="26"/>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="26"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="220" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="199" fontId="69" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="220" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="199" fontId="67" fillId="0" borderId="0" applyFont="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="84" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="221" fontId="85" fillId="0" borderId="0"/>
-    <xf numFmtId="221" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="221" fontId="83" fillId="0" borderId="0"/>
+    <xf numFmtId="221" fontId="83" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="86" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="87" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="84" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="71" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="214" fontId="5" fillId="0" borderId="0" applyFont="0">
       <protection locked="0"/>
     </xf>
@@ -4211,14 +4140,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="22" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="88" fillId="22" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="30" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="22" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="86" fillId="22" borderId="72" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="222" fontId="5" fillId="45" borderId="63">
@@ -4227,16 +4156,16 @@
     <xf numFmtId="223" fontId="5" fillId="45" borderId="73">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="40" fontId="69" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="40" fontId="67" fillId="0" borderId="0" applyFont="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="40" fontId="73" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="40" fontId="71" fillId="0" borderId="0" applyFont="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="224" fontId="89" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="224" fontId="87" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="202" fontId="90" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="202" fontId="88" fillId="0" borderId="0" applyFont="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -4244,18 +4173,18 @@
       <alignment horizontal="right" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="83" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="91" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="89" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="40" fontId="92" fillId="0" borderId="0" applyBorder="0">
+    <xf numFmtId="40" fontId="90" fillId="0" borderId="0" applyBorder="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="202" fontId="69" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="202" fontId="67" fillId="0" borderId="0" applyFont="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="202" fontId="69" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="202" fontId="67" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="199" fontId="10" fillId="48" borderId="0" applyNumberFormat="0" applyAlignment="0">
@@ -4268,58 +4197,58 @@
     <xf numFmtId="228" fontId="5" fillId="45" borderId="63">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="94" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="94" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="199" fontId="95" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="91" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="92" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="92" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="199" fontId="93" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="75" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="75" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="202" fontId="73" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="74" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="75" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="94" fillId="0" borderId="75" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="202" fontId="71" fillId="0" borderId="0"/>
     <xf numFmtId="218" fontId="5" fillId="45" borderId="63">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="229" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="230" fontId="69" fillId="0" borderId="0" applyFill="0">
+    <xf numFmtId="230" fontId="67" fillId="0" borderId="0" applyFill="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="202" fontId="69" fillId="0" borderId="0" applyFont="0">
+    <xf numFmtId="202" fontId="67" fillId="0" borderId="0" applyFont="0">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="187" fontId="82" fillId="0" borderId="8">
+    <xf numFmtId="187" fontId="80" fillId="0" borderId="8">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="82" fillId="0" borderId="8">
+    <xf numFmtId="187" fontId="80" fillId="0" borderId="8">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="54" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="35" applyBorder="0">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
     <xf numFmtId="231" fontId="5" fillId="45" borderId="63">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -4328,7 +4257,7 @@
     </xf>
     <xf numFmtId="40" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="38" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="98" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="96" fillId="0" borderId="0"/>
     <xf numFmtId="194" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="193" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
@@ -4375,7 +4304,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="714">
+  <cellXfs count="715">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -4817,11 +4746,11 @@
     <xf numFmtId="10" fontId="4" fillId="0" borderId="11" xfId="207" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="190"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="190"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="190" applyFont="1"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" xfId="190" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="14" fillId="0" borderId="0" xfId="190" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="171" fontId="6" fillId="0" borderId="11" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4833,7 +4762,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="190" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="190" applyBorder="1"/>
     <xf numFmtId="171" fontId="4" fillId="14" borderId="12" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5063,7 +4992,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="190" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="190" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="190" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="8" xfId="190" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -5072,7 +5001,7 @@
     <xf numFmtId="191" fontId="4" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="16" fillId="0" borderId="0" xfId="190" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="14" fillId="0" borderId="0" xfId="190" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5128,60 +5057,60 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="53" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="55" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="54" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="53" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="52" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="52" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="192" fontId="55" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="192" fontId="53" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="192" fontId="55" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="43" fontId="55" fillId="15" borderId="0" xfId="21" applyFont="1" applyFill="1"/>
-    <xf numFmtId="43" fontId="55" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="55" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="55" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="55" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="55" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="192" fontId="53" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="53" fillId="15" borderId="0" xfId="21" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="53" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="53" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="53" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="55" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="52" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="50" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="57" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="184" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="52" fillId="14" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="50" fillId="14" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="53" fillId="0" borderId="9" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="51" fillId="0" borderId="9" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="99" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="97" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="21"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="21" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="100" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="98" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -5235,18 +5164,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="8" xfId="190" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="54" fillId="15" borderId="0" xfId="21" applyFont="1" applyFill="1"/>
-    <xf numFmtId="43" fontId="54" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="54" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="171" fontId="54" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="101" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="52" fillId="15" borderId="0" xfId="21" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="52" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="52" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="171" fontId="52" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="99" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="54" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="52" fillId="0" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="55" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="54" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="53" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="52" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -5310,7 +5239,7 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="21" applyFont="1"/>
     <xf numFmtId="43" fontId="6" fillId="13" borderId="0" xfId="21" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="192" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="55" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="53" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="4" fillId="7" borderId="9" xfId="184" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="172" fontId="4" fillId="7" borderId="9" xfId="187" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="7" borderId="9" xfId="187" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -5338,23 +5267,23 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="26" xfId="21" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="54" fillId="18" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="52" fillId="18" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="55" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="55" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="53" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="54" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="54" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="52" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="52" fillId="15" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="41" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="52" fillId="0" borderId="9" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="53" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="50" fillId="0" borderId="9" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="22" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5373,16 +5302,16 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="190" applyFont="1"/>
-    <xf numFmtId="43" fontId="52" fillId="0" borderId="0" xfId="21" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="50" fillId="0" borderId="0" xfId="21" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="7" borderId="9" xfId="187" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="82" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="80" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="55" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="55" fillId="0" borderId="0" xfId="21" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="53" fillId="0" borderId="0" xfId="21" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -5397,10 +5326,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="102" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="100" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="102" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="100" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5466,12 +5395,12 @@
     <xf numFmtId="173" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="53" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="4" fillId="7" borderId="8" xfId="21" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="4" fillId="7" borderId="12" xfId="21" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="103" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="101" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="192" applyNumberFormat="1"/>
@@ -5489,22 +5418,22 @@
     <xf numFmtId="14" fontId="0" fillId="49" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="49" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="49" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="102" fillId="49" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="100" fillId="49" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="102" fillId="49" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="100" fillId="49" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="102" fillId="49" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="100" fillId="49" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="102" fillId="49" borderId="17" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="100" fillId="49" borderId="17" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="102" fillId="49" borderId="44" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="100" fillId="49" borderId="44" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="49" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="52" fillId="49" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="14" borderId="8" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -5521,7 +5450,7 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="17" xfId="184" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="18" xfId="184" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="184" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="50" borderId="8" xfId="190" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="50" borderId="8" xfId="190" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="50" borderId="8" xfId="190" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="50" borderId="8" xfId="190" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5591,15 +5520,15 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="102" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="100" fillId="0" borderId="0" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="102" fillId="0" borderId="41" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="100" fillId="0" borderId="41" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -5607,7 +5536,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="102" fillId="49" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="100" fillId="49" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -5758,28 +5687,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -5797,10 +5726,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="33" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5833,10 +5762,10 @@
     <xf numFmtId="167" fontId="4" fillId="0" borderId="9" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5845,13 +5774,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5935,13 +5864,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="25" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5968,26 +5897,29 @@
     <xf numFmtId="167" fontId="6" fillId="0" borderId="50" xfId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="192" fontId="54" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="192" fontId="52" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="54" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="54" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="50" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="48" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="49" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="51" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="184" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1012">
@@ -7503,7 +7435,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet4">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
@@ -12515,7 +12447,7 @@
         <f>+F214</f>
         <v>0</v>
       </c>
-      <c r="G215" s="113">
+      <c r="G215" s="714">
         <f>'Lease Rent'!P99</f>
         <v>2345999.9999999995</v>
       </c>
@@ -12543,7 +12475,7 @@
         <f>+F215*115%</f>
         <v>0</v>
       </c>
-      <c r="G216" s="113">
+      <c r="G216" s="714">
         <f>'Lease Rent'!P103</f>
         <v>781999.99999999988</v>
       </c>
@@ -12948,7 +12880,6 @@
     <customPr name="_pios_id" r:id="rId2"/>
     <customPr name="EpmWorksheetKeyString_GUID" r:id="rId3"/>
   </customProperties>
-  <legacyDrawing r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>